<commit_message>
Cosmetici: contas contábeis por acumulador a partir do Resumo Contábil 01-09/2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GpFQAF7UfcTJUBPm398Z8s
</commit_message>
<xml_diff>
--- a/Cosmetici/Fiscal/2026-09/Acumuladores_Dominio_Cosmetici_2026.xlsx
+++ b/Cosmetici/Fiscal/2026-09/Acumuladores_Dominio_Cosmetici_2026.xlsx
@@ -10,6 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entradas por CFOP" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Saídas por CFOP" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Serviços por prestador" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contas - entradas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contas - saídas e impostos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contas - serviços" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Entradas por CFOP'!$A$4:$G$35</definedName>
@@ -53,7 +56,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -75,6 +78,11 @@
         <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -88,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -98,6 +106,16 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2787,4 +2805,1458 @@
   <autoFilter ref="A4:D40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Contas - entradas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fonte: Resumo Contábil (sintético) do Domínio, 01/01 a 30/09/2026 (pasta 09_2026). Verde = valor fecha exatamente; azul = pelo nome da conta (confirmar); amarelo = não identificado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Acumulador</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>CFOP</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Conta débito</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Conta crédito</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Evidência</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Confiança</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>100 / 101</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>1101 1102 / 2101 2102 2122</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>56 MATÉRIA-PRIMA ou 600 INSUMOS (ICMS: D 30 ICMS A RECUPERAR; IPI: D 29 IPI A RECUPERAR)</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Pelo nome da conta no Resumo Contábil (sem valor que feche) - confirmar. O Resumo tem as duas contas (56: 441.031,19; 600: 84.819,75) e não mostra qual acumulador vai em cada uma</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>104 / 105 / 107</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>1556 / 2556 / 1407</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>513 MATERIAL DE USO E CONSUMO (também aparecem 359 escritório, 360 limpeza/copa, 656 EPI, 58 outros materiais)</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Pelo nome da conta no Resumo Contábil (sem valor que feche) - confirmar. A conta parece ir pelo produto, não só pelo acumulador</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>1411</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>417 (-) DEVOLUÇÃO DE VENDA DE MERCADORIAS</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>504 CLIENTES DIVERSOS (664 COSMETICON quando o cliente é a Cosmeticon)</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Exato: soma do acumulador 02-08/2026 = valor do par no Resumo Contábil 01-09/2026: 390.052,03 = 380.143,70 + 9.908,33</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>133 / 134</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>2202 / 2411</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>415 (-) DEVOLUÇÃO DE VENDA DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>504 CLIENTES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Exato: soma do acumulador 02-08/2026 = valor do par no Resumo Contábil 01-09/2026: 2.312,70 + 10.306,40 = 12.619,10</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>149 / 144</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>1901 / 2901</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>614 ENTRADA P INDUSTRIALIZAÇÃO POR ENCOMENDA</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>607 RETORNO DE MERCADORIA ENVIADA PARA INDUSTRIALIZAÇÃO</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Exato: soma do acumulador 02-08/2026 = valor do par no Resumo Contábil 01-09/2026: 56.948,82 + 16.325,25 = 73.274,07</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>165 / 164</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>1924 / 2924</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>608 REMESSA POR CONTA E ORDEM</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>609 REMESSA POR CONTA E ORDEM</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Exato: soma do acumulador 02-08/2026 = valor do par no Resumo Contábil 01-09/2026: 139.005,39 + 35.347,69 = 174.353,08</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>147 / 148</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>1911 / 2911</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>56 MATÉRIA-PRIMA</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>616 AMOSTRA GRATIS</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Exato: soma do acumulador 02-08/2026 = valor do par no Resumo Contábil 01-09/2026: 37,01 + 156,55 = 193,56</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>2910</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>56 MATÉRIA-PRIMA</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>515 BONIFICAÇÕES RECEBIDAS</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Exato: soma do acumulador 02-08/2026 = valor do par no Resumo Contábil 01-09/2026: 7.550,82</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>1910</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>56 MATÉRIA-PRIMA (provável, igual ao 189)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>515 BONIFICAÇÕES RECEBIDAS</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Sem valor (a única nota foi de R$ 0,00); mesma natureza do 189</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>1949 / 2949</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>612 REMESSA POR EMPRESTIMOS / OUTROS</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>613 REMESSA POR EMPRESTIMOS / OUTROS</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Exato: soma do acumulador 02-08/2026 = valor do par no Resumo Contábil 01-09/2026: 18.410,35</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>198</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>2902</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>607 RETORNO DE MERCADORIA ENVIADA PARA INDUSTRIALIZAÇÃO</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>614 ENTRADA P INDUSTRIALIZAÇÃO POR ENCOMENDA</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Exato: soma do acumulador 02-08/2026 = valor do par no Resumo Contábil 01-09/2026: 41,40</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>199</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>2124</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>618 INDUSTRIALIZAÇÃO EFETUADA POR TERCEIROS</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Exato: soma do acumulador 02-08/2026 = valor do par no Resumo Contábil 01-09/2026: 12.212,04 (Color Way, 02/2026)</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>1000 / 1001</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>1352 1353 1932 / 2352 2353</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>312 FRETES E CARRETOS (ICMS do frete: D 30 ICMS A RECUPERAR)</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS (5 CAIXA GERAL quando à vista)</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Pelo nome da conta no Resumo Contábil (sem valor que feche) - confirmar (312 tem 102.651,91; o Acompanhamento 02-08 soma 47.522,10 - faltam meses/notas no que tenho)</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>192</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>1653</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>não identificado</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Combustível R$ 1.532,52 (03/2026): nenhum par do Resumo fecha</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>238</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>2922</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>não identificado</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>Simples faturamento R$ 5.123,91 (07/2026): nenhum par do Resumo fecha</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>1923</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>não identificado</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr"/>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>CFOP sem histórico em 2026</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>pendente</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Contas - saídas e impostos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fonte: Resumo Contábil (sintético) do Domínio, 01/01 a 30/09/2026 (pasta 09_2026). Verde = valor fecha exatamente; azul = pelo nome da conta (confirmar); amarelo = não identificado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Acumulador / imposto</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>CFOP</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Conta débito</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Conta crédito</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Evidência</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Confiança</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>200 / 201 / 202 / 203</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>5101 5102 / 6101 6102 / 5401 / 6401</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>504 CLIENTES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>408 VENDA DE MERCADORIAS</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Par 504 x 408 no Resumo (1.434.018,14)</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>204 / 205</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>5101 5102 / 5401 (cliente Cosmeticon)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>664 COSMETICON COMERCIO DE COSMETICOS LTDA</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>408 VENDA DE MERCADORIAS</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Par 664 x 408 no Resumo (198.427,30) - conta própria do cliente</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>254 / 255</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>5124 / 6124</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>504 CLIENTES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>411 SERVIÇOS PRESTADOS</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Par 504 x 411 no Resumo (1.615.352,66) - industrialização para terceiros</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>277 / 217</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>5902 / 6902</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>607 RETORNO DE MERCADORIA ENVIADA PARA INDUSTRIALIZAÇÃO</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>614 ENTRADA P INDUSTRIALIZAÇÃO POR ENCOMENDA</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Par 607 x 614 no Resumo (222.207,12)</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>207 / 208</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>5910 / 6910</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>514 BONIFICAÇÕES ENVIADAS</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>55 MERCADORIAS PARA VENDA</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Par 514 x 55 no Resumo (38.503,63)</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>5949</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>612 REMESSA POR EMPRESTIMOS / OUTROS</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>613 REMESSA POR EMPRESTIMOS / OUTROS</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Par 612 x 613 no Resumo (2.354,58)</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>ICMS das saídas</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr"/>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>426 (-) ICMS</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>172 ICMS A RECOLHER</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Par do Resumo Contábil</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>ICMS-ST das saídas</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr"/>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>482 (-) SUBSTITUIÇÃO TRIBUTÁRIA</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>481 SUBSTITUIÇÃO TRIBUTÁRIA A RECOLHER</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Par do Resumo Contábil</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>IPI das saídas</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr"/>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>425 (-) IPI</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>171 IPI A RECOLHER</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Par do Resumo Contábil</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>PIS</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr"/>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>429 (-) PIS</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>179 PIS A RECOLHER</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Par do Resumo Contábil</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>COFINS</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr"/>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>428 (-) COFINS</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>180 COFINS A RECOLHER</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Par do Resumo Contábil</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>CSLL</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr"/>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>477 (-) CONTRIBUIÇÃO SOCIAL</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>177 CONTRIBUIÇÃO SOCIAL A RECOLHER</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Par do Resumo Contábil</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>IRPJ</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr"/>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>478 (-) IMPOSTO DE RENDA</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>176 IMPOSTO DE RENDA A RECOLHER</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Par do Resumo Contábil</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>ICMS das entradas (crédito)</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr"/>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>30 ICMS A RECUPERAR</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>conta da mercadoria / frete (56, 312, 618, 612...)</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Par do Resumo Contábil</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>IPI das entradas (crédito)</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr"/>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>29 IPI A RECUPERAR</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>56 MATÉRIA-PRIMA</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Par do Resumo Contábil</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Apuração ICMS / IPI</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr"/>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>172 ICMS A RECOLHER / 171 IPI A RECOLHER</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>30 ICMS A RECUPERAR / 29 IPI A RECUPERAR</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Par do Resumo Contábil</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>DIFAL (uso e consumo de fora)</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr"/>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>527 ICMS DIFERENCIAL DE ALIQUOTA</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>526 ICMS DIF. DE ALIQUOTA A RECOLHER (crédito: D 30 / C 527)</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Par do Resumo Contábil</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>ISS retido nas NFS-e tomadas</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr"/>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>183 ISS RETIDO A RECOLHER</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Par do Resumo Contábil</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>IRRF retido nas NFS-e tomadas</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr"/>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>178 IRRF A RECOLHER</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>Par do Resumo Contábil</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Contas - serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serviços tomados: o Resumo sintético não liga a conta ao prestador. Contas de despesa que aparecem contra 506 FORNECEDORES - o vínculo com o acumulador é provável, não confirmado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Conta débito</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Conta crédito</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Valor 01-09/2026 e acumulador provável</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>361 ASSISTÊNCIA CONTÁBIL</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>510 HONORÁRIOS CONTÁBEIS A PAGAR</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>17.000,00 - provável 828 (Protection Assessoria)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>362 SERVIÇOS PRESTADOS POR TERCEIROS</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>82.167,16 + 10.498,65 (com retenção)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>364 DESPESAS ADMINISTRATIVAS</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>149.107,61 - provável 816 (Flash, créditos de benefícios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>640 SOFTWARE/SISTEMA</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>24.723,54 - provável 811 CRM, 818 Nextar, 823 Tecnoponto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>576 PLANO DE SAÚDE EMPREGADOS</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>5.188,40 - provável 824 Dental Uni, 821 Plus Santé</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>652 ASSISTENCIA MÉDICA E SOCIAL</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>1.344,50 - provável 831 CMS / 832 Interclin (medicina do trabalho)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>627 DESPESAS LABORATORIAIS</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>1.178,00 - provável 810 Bioactive / Kosmoscience</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>643 PROPAGANDA</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>1.567,76 - provável 830 gráficas</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>325 SERVIÇOS PRESTADOS POR TERCEIROS (custo)</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>2.405,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>321 MANUTENÇÃO E REPARO</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>608,39</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>715 HONORARIOS ADVOCATICIOS</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>1.500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>618 INDUSTRIALIZAÇÃO EFETUADA POR TERCEIROS</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>506 FORNECEDORES DIVERSOS</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>12.212,04 (acumulador 199)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>